<commit_message>
Refactor database connection handling and improve WSGI app loading
- Updated config.py to strip whitespace from DATABASE_URL to prevent connection issues with PostgreSQL.
- Enhanced Injaaz.py with improved retry logic for database connections, ensuring timely retries and logging.
- Modified wsgi.py to implement a deferred loading mechanism for the Flask app, allowing for better handling of connection timeouts during deployment.
- Adjusted render.yaml to prevent issues with gunicorn's --preload option, ensuring the app binds to the correct port.
- Incremented version numbers for relevant files to reflect recent changes.
</commit_message>
<xml_diff>
--- a/\\172.25.70.143\Injaaz\General\CAFM/Daily Report on Resolved and Pending Complaints for 15th of July 2026 & 16th of July 2026.xlsx
+++ b/\\172.25.70.143\Injaaz\General\CAFM/Daily Report on Resolved and Pending Complaints for 15th of July 2026 & 16th of July 2026.xlsx
@@ -999,7 +999,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:10</t>
+          <t>Generated: 05 Sep 2026  21:47</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:10</t>
+          <t>Generated: 05 Sep 2026  21:47</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:10</t>
+          <t>Generated: 05 Sep 2026  21:47</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:10</t>
+          <t>Generated: 05 Sep 2026  21:47</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2104,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:10</t>
+          <t>Generated: 05 Sep 2026  21:47</t>
         </is>
       </c>
     </row>

</xml_diff>